<commit_message>
fix(pivots): reference generator — x14 cache ext URI, template-shaped seed pivot (Task 2 fix round 2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KTccUzeFqqMqTthqgFm9H
</commit_message>
<xml_diff>
--- a/tests/fixtures/xlsx-pivots/slicer-dark1.xlsx
+++ b/tests/fixtures/xlsx-pivots/slicer-dark1.xlsx
@@ -257,9 +257,9 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" recordCount="16" refreshOnLoad="1" saveData="1">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" recordCount="40" refreshOnLoad="1" saveData="1">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:E17" sheet="Data"/>
+    <worksheetSource ref="A1:E41" sheet="Data"/>
   </cacheSource>
   <cacheFields count="5">
     <cacheField name="Region">
@@ -278,28 +278,51 @@
         <s v="Cherries"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Date">
-      <sharedItems containsDate="1" containsNonDate="0" count="16">
-        <d v="2024-05-22T00:00:00Z"/>
-        <d v="2025-04-13T00:00:00Z"/>
-        <d v="2024-12-10T00:00:00Z"/>
-        <d v="2024-08-02T00:00:00Z"/>
-        <d v="2025-12-02T00:00:00Z"/>
-        <d v="2025-05-03T00:00:00Z"/>
-        <d v="2024-01-05T00:00:00Z"/>
-        <d v="2024-05-18T00:00:00Z"/>
-        <d v="2025-01-28T00:00:00Z"/>
-        <d v="2025-01-15T00:00:00Z"/>
-        <d v="2025-05-14T00:00:00Z"/>
-        <d v="2025-07-04T00:00:00Z"/>
-        <d v="2024-03-31T00:00:00Z"/>
-        <d v="2025-06-04T00:00:00Z"/>
-        <d v="2024-11-12T00:00:00Z"/>
-        <d v="2024-01-16T00:00:00Z"/>
+    <cacheField name="Date" numFmtId="176">
+      <sharedItems containsDate="1" containsNonDate="0" count="39">
+        <d v="2024-01-12T00:00:00"/>
+        <d v="2024-01-13T00:00:00"/>
+        <d v="2024-01-14T00:00:00"/>
+        <d v="2024-01-15T00:00:00"/>
+        <d v="2024-01-16T00:00:00"/>
+        <d v="2024-01-17T00:00:00"/>
+        <d v="2024-01-18T00:00:00"/>
+        <d v="2024-01-19T00:00:00"/>
+        <d v="2024-01-20T00:00:00"/>
+        <d v="2024-01-21T00:00:00"/>
+        <d v="2024-01-22T00:00:00"/>
+        <d v="2024-01-23T00:00:00"/>
+        <d v="2024-01-24T00:00:00"/>
+        <d v="2024-01-25T00:00:00"/>
+        <d v="2024-01-26T00:00:00"/>
+        <d v="2024-01-27T00:00:00"/>
+        <d v="2024-01-28T00:00:00"/>
+        <d v="2024-01-29T00:00:00"/>
+        <d v="2024-01-30T00:00:00"/>
+        <d v="2024-01-31T00:00:00"/>
+        <d v="2024-02-01T00:00:00"/>
+        <d v="2024-02-02T00:00:00"/>
+        <d v="2024-02-03T00:00:00"/>
+        <d v="2024-02-04T00:00:00"/>
+        <d v="2024-02-05T00:00:00"/>
+        <d v="2024-02-06T00:00:00"/>
+        <d v="2024-02-07T00:00:00"/>
+        <d v="2024-02-08T00:00:00"/>
+        <d v="2024-02-09T00:00:00"/>
+        <d v="2024-02-10T00:00:00"/>
+        <d v="2024-02-11T00:00:00"/>
+        <d v="2024-02-12T00:00:00"/>
+        <d v="2024-02-13T00:00:00"/>
+        <d v="2024-02-14T00:00:00"/>
+        <d v="2024-02-15T00:00:00"/>
+        <d v="2024-02-16T00:00:00"/>
+        <d v="2024-02-17T00:00:00"/>
+        <d v="2024-02-18T00:00:00"/>
+        <d v="2024-02-19T00:00:00"/>
       </sharedItems>
     </cacheField>
     <cacheField name="Sales">
-      <sharedItems count="16">
+      <sharedItems count="40">
         <n v="6799"/>
         <n v="2066.01"/>
         <n v="1649.02"/>
@@ -316,10 +339,34 @@
         <n v="1742.13"/>
         <n v="4053.14"/>
         <n v="952.15"/>
+        <n v="1311.16"/>
+        <n v="7522.17"/>
+        <n v="3441.18"/>
+        <n v="1836.19"/>
+        <n v="8291.2"/>
+        <n v="2902.21"/>
+        <n v="949.22"/>
+        <n v="6032.23"/>
+        <n v="2639.24"/>
+        <n v="810.25"/>
+        <n v="3745.26"/>
+        <n v="5716.27"/>
+        <n v="8699.28"/>
+        <n v="5630.29"/>
+        <n v="4877.3"/>
+        <n v="3568.31"/>
+        <n v="8711.32"/>
+        <n v="1058.33"/>
+        <n v="1897.34"/>
+        <n v="4548.35"/>
+        <n v="6731.36"/>
+        <n v="2902.37"/>
+        <n v="6653.38"/>
+        <n v="5456.39"/>
       </sharedItems>
     </cacheField>
     <cacheField name="Units">
-      <sharedItems count="14">
+      <sharedItems count="33">
         <n v="71"/>
         <n v="68"/>
         <n v="63"/>
@@ -334,11 +381,30 @@
         <n v="84"/>
         <n v="41"/>
         <n v="66"/>
+        <n v="25"/>
+        <n v="2"/>
+        <n v="21"/>
+        <n v="8"/>
+        <n v="81"/>
+        <n v="86"/>
+        <n v="51"/>
+        <n v="53"/>
+        <n v="87"/>
+        <n v="24"/>
+        <n v="37"/>
+        <n v="54"/>
+        <n v="77"/>
+        <n v="22"/>
+        <n v="69"/>
+        <n v="82"/>
+        <n v="61"/>
+        <n v="15"/>
+        <n v="50"/>
       </sharedItems>
     </cacheField>
   </cacheFields>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
       <x14:pivotCacheDefinition pivotCacheId="1" slicerData="1"/>
     </ext>
   </extLst>
@@ -346,7 +412,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16">
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40">
   <r>
     <x v="0"/>
     <x v="0"/>
@@ -458,52 +524,253 @@
     <x v="15"/>
     <x v="15"/>
     <x v="13"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="16"/>
+    <x v="16"/>
+    <x v="14"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="17"/>
+    <x v="17"/>
+    <x v="15"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="18"/>
+    <x v="18"/>
+    <x v="16"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="19"/>
+    <x v="19"/>
+    <x v="17"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="20"/>
+    <x v="20"/>
+    <x v="18"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="21"/>
+    <x v="21"/>
+    <x v="19"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="22"/>
+    <x v="22"/>
+    <x v="20"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="23"/>
+    <x v="23"/>
+    <x v="13"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="24"/>
+    <x v="24"/>
+    <x v="21"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="25"/>
+    <x v="25"/>
+    <x v="13"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="26"/>
+    <x v="26"/>
+    <x v="22"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="27"/>
+    <x v="27"/>
+    <x v="23"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="28"/>
+    <x v="28"/>
+    <x v="24"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="29"/>
+    <x v="29"/>
+    <x v="25"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="30"/>
+    <x v="30"/>
+    <x v="26"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="31"/>
+    <x v="31"/>
+    <x v="27"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="32"/>
+    <x v="32"/>
+    <x v="12"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="33"/>
+    <x v="33"/>
+    <x v="25"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="34"/>
+    <x v="34"/>
+    <x v="28"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="35"/>
+    <x v="35"/>
+    <x v="29"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <x v="0"/>
+    <x v="36"/>
+    <x v="36"/>
+    <x v="30"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="37"/>
+    <x v="37"/>
+    <x v="15"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="38"/>
+    <x v="38"/>
+    <x v="31"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="0"/>
+    <x v="39"/>
+    <x v="32"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PivotTable1" cacheId="1" dataCaption="Values" compact="1" outline="1" subtotalTop="1">
-  <location ref="G1:H6" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+  <location ref="G1:H6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">
-      <items count="4">
+      <items count="5">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
+        <item t="default"/>
       </items>
     </pivotField>
     <pivotField showAll="0">
-      <items count="4">
+      <items count="5">
+        <item x="2"/>
+        <item h="1" x="1"/>
+        <item x="3"/>
+        <item h="1" x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField numFmtId="176" showAll="0">
+      <items count="40">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
         <item x="3"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="1">
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="34"/>
+        <item x="35"/>
+        <item x="36"/>
+        <item x="37"/>
+        <item x="38"/>
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField dataField="1" showAll="0">
-      <items count="1">
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="1">
-        <item t="default"/>
-      </items>
-    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
     <field x="0"/>
   </rowFields>
-  <rowItems count="4">
+  <rowItems count="5">
     <i>
-      <x v="0"/>
+      <x/>
     </i>
     <i>
       <x v="1"/>
@@ -514,11 +781,25 @@
     <i>
       <x v="3"/>
     </i>
+    <i t="grand">
+      <x/>
+    </i>
   </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
   <dataFields count="1">
     <dataField name="Sum of Sales" fld="3" subtotal="sum"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="1" showColStripes="0"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
 </pivotTableDefinition>
 </file>
 
@@ -673,7 +954,7 @@
         </is>
       </c>
       <c r="H2">
-        <v>14896.359999999999</v>
+        <v>42054.1</v>
       </c>
     </row>
     <row r="3">
@@ -683,7 +964,7 @@
         </is>
       </c>
       <c r="H3">
-        <v>14852.32</v>
+        <v>36416</v>
       </c>
     </row>
     <row r="4">
@@ -693,7 +974,7 @@
         </is>
       </c>
       <c r="H4">
-        <v>13528.280000000002</v>
+        <v>34353.90000000001</v>
       </c>
     </row>
     <row r="5">
@@ -703,7 +984,7 @@
         </is>
       </c>
       <c r="H5">
-        <v>28788.24</v>
+        <v>65171.8</v>
       </c>
     </row>
     <row r="6">
@@ -713,7 +994,7 @@
         </is>
       </c>
       <c r="H6">
-        <v>72065.2</v>
+        <v>177995.8</v>
       </c>
     </row>
   </sheetData>
@@ -737,7 +1018,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -779,7 +1060,7 @@
         </is>
       </c>
       <c r="C2" s="2">
-        <v>45434</v>
+        <v>45303</v>
       </c>
       <c r="D2">
         <v>6799</v>
@@ -800,7 +1081,7 @@
         </is>
       </c>
       <c r="C3" s="2">
-        <v>45760</v>
+        <v>45304</v>
       </c>
       <c r="D3">
         <v>2066.01</v>
@@ -821,7 +1102,7 @@
         </is>
       </c>
       <c r="C4" s="2">
-        <v>45636</v>
+        <v>45305</v>
       </c>
       <c r="D4">
         <v>1649.02</v>
@@ -842,7 +1123,7 @@
         </is>
       </c>
       <c r="C5" s="2">
-        <v>45506</v>
+        <v>45306</v>
       </c>
       <c r="D5">
         <v>3500.03</v>
@@ -863,7 +1144,7 @@
         </is>
       </c>
       <c r="C6" s="2">
-        <v>45993</v>
+        <v>45307</v>
       </c>
       <c r="D6">
         <v>7923.04</v>
@@ -884,7 +1165,7 @@
         </is>
       </c>
       <c r="C7" s="2">
-        <v>45780</v>
+        <v>45308</v>
       </c>
       <c r="D7">
         <v>766.05</v>
@@ -905,7 +1186,7 @@
         </is>
       </c>
       <c r="C8" s="2">
-        <v>45296</v>
+        <v>45309</v>
       </c>
       <c r="D8">
         <v>2277.06</v>
@@ -926,7 +1207,7 @@
         </is>
       </c>
       <c r="C9" s="2">
-        <v>45430</v>
+        <v>45310</v>
       </c>
       <c r="D9">
         <v>2560.07</v>
@@ -947,7 +1228,7 @@
         </is>
       </c>
       <c r="C10" s="2">
-        <v>45685</v>
+        <v>45311</v>
       </c>
       <c r="D10">
         <v>6655.08</v>
@@ -968,7 +1249,7 @@
         </is>
       </c>
       <c r="C11" s="2">
-        <v>45672</v>
+        <v>45312</v>
       </c>
       <c r="D11">
         <v>8954.09</v>
@@ -989,7 +1270,7 @@
         </is>
       </c>
       <c r="C12" s="2">
-        <v>45791</v>
+        <v>45313</v>
       </c>
       <c r="D12">
         <v>6873.1</v>
@@ -1010,7 +1291,7 @@
         </is>
       </c>
       <c r="C13" s="2">
-        <v>45842</v>
+        <v>45314</v>
       </c>
       <c r="D13">
         <v>7884.11</v>
@@ -1031,7 +1312,7 @@
         </is>
       </c>
       <c r="C14" s="2">
-        <v>45382</v>
+        <v>45315</v>
       </c>
       <c r="D14">
         <v>7411.12</v>
@@ -1052,7 +1333,7 @@
         </is>
       </c>
       <c r="C15" s="2">
-        <v>45812</v>
+        <v>45316</v>
       </c>
       <c r="D15">
         <v>1742.13</v>
@@ -1073,7 +1354,7 @@
         </is>
       </c>
       <c r="C16" s="2">
-        <v>45608</v>
+        <v>45317</v>
       </c>
       <c r="D16">
         <v>4053.14</v>
@@ -1094,13 +1375,517 @@
         </is>
       </c>
       <c r="C17" s="2">
-        <v>45307</v>
+        <v>45318</v>
       </c>
       <c r="D17">
         <v>952.15</v>
       </c>
       <c r="E17">
         <v>66</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Bananas</t>
+        </is>
+      </c>
+      <c r="C18" s="2">
+        <v>45319</v>
+      </c>
+      <c r="D18">
+        <v>1311.16</v>
+      </c>
+      <c r="E18">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Dates</t>
+        </is>
+      </c>
+      <c r="C19" s="2">
+        <v>45320</v>
+      </c>
+      <c r="D19">
+        <v>7522.17</v>
+      </c>
+      <c r="E19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Apples</t>
+        </is>
+      </c>
+      <c r="C20" s="2">
+        <v>45321</v>
+      </c>
+      <c r="D20">
+        <v>3441.18</v>
+      </c>
+      <c r="E20">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Cherries</t>
+        </is>
+      </c>
+      <c r="C21" s="2">
+        <v>45322</v>
+      </c>
+      <c r="D21">
+        <v>1836.19</v>
+      </c>
+      <c r="E21">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Bananas</t>
+        </is>
+      </c>
+      <c r="C22" s="2">
+        <v>45323</v>
+      </c>
+      <c r="D22">
+        <v>8291.2</v>
+      </c>
+      <c r="E22">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Dates</t>
+        </is>
+      </c>
+      <c r="C23" s="2">
+        <v>45324</v>
+      </c>
+      <c r="D23">
+        <v>2902.21</v>
+      </c>
+      <c r="E23">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Apples</t>
+        </is>
+      </c>
+      <c r="C24" s="2">
+        <v>45325</v>
+      </c>
+      <c r="D24">
+        <v>949.22</v>
+      </c>
+      <c r="E24">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Cherries</t>
+        </is>
+      </c>
+      <c r="C25" s="2">
+        <v>45326</v>
+      </c>
+      <c r="D25">
+        <v>6032.23</v>
+      </c>
+      <c r="E25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Bananas</t>
+        </is>
+      </c>
+      <c r="C26" s="2">
+        <v>45327</v>
+      </c>
+      <c r="D26">
+        <v>2639.24</v>
+      </c>
+      <c r="E26">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Dates</t>
+        </is>
+      </c>
+      <c r="C27" s="2">
+        <v>45328</v>
+      </c>
+      <c r="D27">
+        <v>810.25</v>
+      </c>
+      <c r="E27">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Apples</t>
+        </is>
+      </c>
+      <c r="C28" s="2">
+        <v>45329</v>
+      </c>
+      <c r="D28">
+        <v>3745.26</v>
+      </c>
+      <c r="E28">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Cherries</t>
+        </is>
+      </c>
+      <c r="C29" s="2">
+        <v>45330</v>
+      </c>
+      <c r="D29">
+        <v>5716.27</v>
+      </c>
+      <c r="E29">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Bananas</t>
+        </is>
+      </c>
+      <c r="C30" s="2">
+        <v>45331</v>
+      </c>
+      <c r="D30">
+        <v>8699.28</v>
+      </c>
+      <c r="E30">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Dates</t>
+        </is>
+      </c>
+      <c r="C31" s="2">
+        <v>45332</v>
+      </c>
+      <c r="D31">
+        <v>5630.29</v>
+      </c>
+      <c r="E31">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Apples</t>
+        </is>
+      </c>
+      <c r="C32" s="2">
+        <v>45333</v>
+      </c>
+      <c r="D32">
+        <v>4877.3</v>
+      </c>
+      <c r="E32">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Cherries</t>
+        </is>
+      </c>
+      <c r="C33" s="2">
+        <v>45334</v>
+      </c>
+      <c r="D33">
+        <v>3568.31</v>
+      </c>
+      <c r="E33">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Bananas</t>
+        </is>
+      </c>
+      <c r="C34" s="2">
+        <v>45335</v>
+      </c>
+      <c r="D34">
+        <v>8711.32</v>
+      </c>
+      <c r="E34">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Dates</t>
+        </is>
+      </c>
+      <c r="C35" s="2">
+        <v>45336</v>
+      </c>
+      <c r="D35">
+        <v>1058.33</v>
+      </c>
+      <c r="E35">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Apples</t>
+        </is>
+      </c>
+      <c r="C36" s="2">
+        <v>45337</v>
+      </c>
+      <c r="D36">
+        <v>1897.34</v>
+      </c>
+      <c r="E36">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Cherries</t>
+        </is>
+      </c>
+      <c r="C37" s="2">
+        <v>45338</v>
+      </c>
+      <c r="D37">
+        <v>4548.35</v>
+      </c>
+      <c r="E37">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Bananas</t>
+        </is>
+      </c>
+      <c r="C38" s="2">
+        <v>45339</v>
+      </c>
+      <c r="D38">
+        <v>6731.36</v>
+      </c>
+      <c r="E38">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Dates</t>
+        </is>
+      </c>
+      <c r="C39" s="2">
+        <v>45340</v>
+      </c>
+      <c r="D39">
+        <v>2902.37</v>
+      </c>
+      <c r="E39">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Apples</t>
+        </is>
+      </c>
+      <c r="C40" s="2">
+        <v>45341</v>
+      </c>
+      <c r="D40">
+        <v>6653.38</v>
+      </c>
+      <c r="E40">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Cherries</t>
+        </is>
+      </c>
+      <c r="C41" s="2">
+        <v>45303</v>
+      </c>
+      <c r="D41">
+        <v>5456.39</v>
+      </c>
+      <c r="E41">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(pivots): reference generator — Excel-accepted cache shape (versions, type flags, inline numerics, no slicerData) (Task 2 fix round 3)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KTccUzeFqqMqTthqgFm9H
</commit_message>
<xml_diff>
--- a/tests/fixtures/xlsx-pivots/slicer-dark1.xlsx
+++ b/tests/fixtures/xlsx-pivots/slicer-dark1.xlsx
@@ -257,12 +257,12 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" recordCount="40" refreshOnLoad="1" saveData="1">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="40" saveData="1">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:E41" sheet="Data"/>
   </cacheSource>
   <cacheFields count="5">
-    <cacheField name="Region">
+    <cacheField name="Region" numFmtId="0">
       <sharedItems count="4">
         <s v="South"/>
         <s v="North"/>
@@ -270,7 +270,7 @@
         <s v="East"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Product">
+    <cacheField name="Product" numFmtId="0">
       <sharedItems count="4">
         <s v="Bananas"/>
         <s v="Dates"/>
@@ -279,7 +279,7 @@
       </sharedItems>
     </cacheField>
     <cacheField name="Date" numFmtId="176">
-      <sharedItems containsDate="1" containsNonDate="0" count="39">
+      <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2024-01-12T00:00:00" maxDate="2024-02-19T00:00:00" count="39">
         <d v="2024-01-12T00:00:00"/>
         <d v="2024-01-13T00:00:00"/>
         <d v="2024-01-14T00:00:00"/>
@@ -321,91 +321,16 @@
         <d v="2024-02-19T00:00:00"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="Sales">
-      <sharedItems count="40">
-        <n v="6799"/>
-        <n v="2066.01"/>
-        <n v="1649.02"/>
-        <n v="3500.03"/>
-        <n v="7923.04"/>
-        <n v="766.05"/>
-        <n v="2277.06"/>
-        <n v="2560.07"/>
-        <n v="6655.08"/>
-        <n v="8954.09"/>
-        <n v="6873.1"/>
-        <n v="7884.11"/>
-        <n v="7411.12"/>
-        <n v="1742.13"/>
-        <n v="4053.14"/>
-        <n v="952.15"/>
-        <n v="1311.16"/>
-        <n v="7522.17"/>
-        <n v="3441.18"/>
-        <n v="1836.19"/>
-        <n v="8291.2"/>
-        <n v="2902.21"/>
-        <n v="949.22"/>
-        <n v="6032.23"/>
-        <n v="2639.24"/>
-        <n v="810.25"/>
-        <n v="3745.26"/>
-        <n v="5716.27"/>
-        <n v="8699.28"/>
-        <n v="5630.29"/>
-        <n v="4877.3"/>
-        <n v="3568.31"/>
-        <n v="8711.32"/>
-        <n v="1058.33"/>
-        <n v="1897.34"/>
-        <n v="4548.35"/>
-        <n v="6731.36"/>
-        <n v="2902.37"/>
-        <n v="6653.38"/>
-        <n v="5456.39"/>
-      </sharedItems>
+    <cacheField name="Sales" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="766.05" maxValue="8954.09"/>
     </cacheField>
-    <cacheField name="Units">
-      <sharedItems count="33">
-        <n v="71"/>
-        <n v="68"/>
-        <n v="63"/>
-        <n v="70"/>
-        <n v="7"/>
-        <n v="32"/>
-        <n v="34"/>
-        <n v="3"/>
-        <n v="72"/>
-        <n v="80"/>
-        <n v="59"/>
-        <n v="84"/>
-        <n v="41"/>
-        <n v="66"/>
-        <n v="25"/>
-        <n v="2"/>
-        <n v="21"/>
-        <n v="8"/>
-        <n v="81"/>
-        <n v="86"/>
-        <n v="51"/>
-        <n v="53"/>
-        <n v="87"/>
-        <n v="24"/>
-        <n v="37"/>
-        <n v="54"/>
-        <n v="77"/>
-        <n v="22"/>
-        <n v="69"/>
-        <n v="82"/>
-        <n v="61"/>
-        <n v="15"/>
-        <n v="50"/>
-      </sharedItems>
+    <cacheField name="Units" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="2" maxValue="87"/>
     </cacheField>
   </cacheFields>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition pivotCacheId="1" slicerData="1"/>
+      <x14:pivotCacheDefinition pivotCacheId="1"/>
     </ext>
   </extLst>
 </pivotCacheDefinition>
@@ -417,287 +342,287 @@
     <x v="0"/>
     <x v="0"/>
     <x v="0"/>
-    <x v="0"/>
-    <x v="0"/>
-  </r>
-  <r>
-    <x v="1"/>
-    <x v="1"/>
-    <x v="1"/>
-    <x v="1"/>
-    <x v="1"/>
-  </r>
-  <r>
-    <x v="2"/>
-    <x v="2"/>
-    <x v="2"/>
-    <x v="2"/>
-    <x v="2"/>
-  </r>
-  <r>
-    <x v="3"/>
-    <x v="3"/>
-    <x v="3"/>
-    <x v="3"/>
-    <x v="3"/>
+    <n v="6799"/>
+    <n v="71"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <x v="1"/>
+    <x v="1"/>
+    <n v="2066.01"/>
+    <n v="68"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <x v="2"/>
+    <x v="2"/>
+    <n v="1649.02"/>
+    <n v="63"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="3"/>
+    <n v="3500.03"/>
+    <n v="70"/>
   </r>
   <r>
     <x v="0"/>
     <x v="0"/>
     <x v="4"/>
-    <x v="4"/>
-    <x v="4"/>
+    <n v="7923.04"/>
+    <n v="7"/>
   </r>
   <r>
     <x v="1"/>
     <x v="1"/>
     <x v="5"/>
-    <x v="5"/>
-    <x v="5"/>
+    <n v="766.05"/>
+    <n v="32"/>
   </r>
   <r>
     <x v="2"/>
     <x v="2"/>
     <x v="6"/>
-    <x v="6"/>
-    <x v="0"/>
+    <n v="2277.06"/>
+    <n v="71"/>
   </r>
   <r>
     <x v="3"/>
     <x v="3"/>
     <x v="7"/>
-    <x v="7"/>
-    <x v="6"/>
+    <n v="2560.07"/>
+    <n v="34"/>
   </r>
   <r>
     <x v="0"/>
     <x v="0"/>
     <x v="8"/>
-    <x v="8"/>
-    <x v="7"/>
+    <n v="6655.08"/>
+    <n v="3"/>
   </r>
   <r>
     <x v="1"/>
     <x v="1"/>
     <x v="9"/>
-    <x v="9"/>
-    <x v="8"/>
+    <n v="8954.09"/>
+    <n v="72"/>
   </r>
   <r>
     <x v="2"/>
     <x v="2"/>
     <x v="10"/>
-    <x v="10"/>
-    <x v="7"/>
+    <n v="6873.1"/>
+    <n v="3"/>
   </r>
   <r>
     <x v="3"/>
     <x v="3"/>
     <x v="11"/>
-    <x v="11"/>
-    <x v="9"/>
+    <n v="7884.11"/>
+    <n v="80"/>
   </r>
   <r>
     <x v="0"/>
     <x v="0"/>
     <x v="12"/>
-    <x v="12"/>
-    <x v="10"/>
+    <n v="7411.12"/>
+    <n v="59"/>
   </r>
   <r>
     <x v="1"/>
     <x v="1"/>
     <x v="13"/>
-    <x v="13"/>
-    <x v="11"/>
+    <n v="1742.13"/>
+    <n v="84"/>
   </r>
   <r>
     <x v="2"/>
     <x v="2"/>
     <x v="14"/>
-    <x v="14"/>
-    <x v="12"/>
+    <n v="4053.14"/>
+    <n v="41"/>
   </r>
   <r>
     <x v="3"/>
     <x v="3"/>
     <x v="15"/>
-    <x v="15"/>
-    <x v="13"/>
+    <n v="952.15"/>
+    <n v="66"/>
   </r>
   <r>
     <x v="0"/>
     <x v="0"/>
     <x v="16"/>
-    <x v="16"/>
-    <x v="14"/>
+    <n v="1311.16"/>
+    <n v="25"/>
   </r>
   <r>
     <x v="1"/>
     <x v="1"/>
     <x v="17"/>
-    <x v="17"/>
-    <x v="15"/>
+    <n v="7522.17"/>
+    <n v="2"/>
   </r>
   <r>
     <x v="2"/>
     <x v="2"/>
     <x v="18"/>
-    <x v="18"/>
-    <x v="16"/>
+    <n v="3441.18"/>
+    <n v="21"/>
   </r>
   <r>
     <x v="3"/>
     <x v="3"/>
     <x v="19"/>
-    <x v="19"/>
-    <x v="17"/>
+    <n v="1836.19"/>
+    <n v="8"/>
   </r>
   <r>
     <x v="0"/>
     <x v="0"/>
     <x v="20"/>
-    <x v="20"/>
-    <x v="18"/>
+    <n v="8291.2"/>
+    <n v="81"/>
   </r>
   <r>
     <x v="1"/>
     <x v="1"/>
     <x v="21"/>
-    <x v="21"/>
-    <x v="19"/>
+    <n v="2902.21"/>
+    <n v="86"/>
   </r>
   <r>
     <x v="2"/>
     <x v="2"/>
     <x v="22"/>
-    <x v="22"/>
-    <x v="20"/>
+    <n v="949.22"/>
+    <n v="51"/>
   </r>
   <r>
     <x v="3"/>
     <x v="3"/>
     <x v="23"/>
-    <x v="23"/>
-    <x v="13"/>
+    <n v="6032.23"/>
+    <n v="66"/>
   </r>
   <r>
     <x v="0"/>
     <x v="0"/>
     <x v="24"/>
-    <x v="24"/>
-    <x v="21"/>
+    <n v="2639.24"/>
+    <n v="53"/>
   </r>
   <r>
     <x v="1"/>
     <x v="1"/>
     <x v="25"/>
-    <x v="25"/>
-    <x v="13"/>
+    <n v="810.25"/>
+    <n v="66"/>
   </r>
   <r>
     <x v="2"/>
     <x v="2"/>
     <x v="26"/>
-    <x v="26"/>
-    <x v="22"/>
+    <n v="3745.26"/>
+    <n v="87"/>
   </r>
   <r>
     <x v="3"/>
     <x v="3"/>
     <x v="27"/>
-    <x v="27"/>
-    <x v="23"/>
+    <n v="5716.27"/>
+    <n v="24"/>
   </r>
   <r>
     <x v="0"/>
     <x v="0"/>
     <x v="28"/>
-    <x v="28"/>
-    <x v="24"/>
+    <n v="8699.28"/>
+    <n v="37"/>
   </r>
   <r>
     <x v="1"/>
     <x v="1"/>
     <x v="29"/>
-    <x v="29"/>
-    <x v="25"/>
+    <n v="5630.29"/>
+    <n v="54"/>
   </r>
   <r>
     <x v="2"/>
     <x v="2"/>
     <x v="30"/>
-    <x v="30"/>
-    <x v="26"/>
+    <n v="4877.3"/>
+    <n v="77"/>
   </r>
   <r>
     <x v="3"/>
     <x v="3"/>
     <x v="31"/>
-    <x v="31"/>
-    <x v="27"/>
+    <n v="3568.31"/>
+    <n v="22"/>
   </r>
   <r>
     <x v="0"/>
     <x v="0"/>
     <x v="32"/>
-    <x v="32"/>
-    <x v="12"/>
+    <n v="8711.32"/>
+    <n v="41"/>
   </r>
   <r>
     <x v="1"/>
     <x v="1"/>
     <x v="33"/>
-    <x v="33"/>
-    <x v="25"/>
+    <n v="1058.33"/>
+    <n v="54"/>
   </r>
   <r>
     <x v="2"/>
     <x v="2"/>
     <x v="34"/>
-    <x v="34"/>
-    <x v="28"/>
+    <n v="1897.34"/>
+    <n v="69"/>
   </r>
   <r>
     <x v="3"/>
     <x v="3"/>
     <x v="35"/>
-    <x v="35"/>
-    <x v="29"/>
+    <n v="4548.35"/>
+    <n v="82"/>
   </r>
   <r>
     <x v="0"/>
     <x v="0"/>
     <x v="36"/>
-    <x v="36"/>
-    <x v="30"/>
+    <n v="6731.36"/>
+    <n v="61"/>
   </r>
   <r>
     <x v="1"/>
     <x v="1"/>
     <x v="37"/>
-    <x v="37"/>
-    <x v="15"/>
+    <n v="2902.37"/>
+    <n v="2"/>
   </r>
   <r>
     <x v="2"/>
     <x v="2"/>
     <x v="38"/>
-    <x v="38"/>
-    <x v="31"/>
-  </r>
-  <r>
-    <x v="3"/>
-    <x v="3"/>
-    <x v="0"/>
-    <x v="39"/>
-    <x v="32"/>
+    <n v="6653.38"/>
+    <n v="15"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <x v="3"/>
+    <x v="0"/>
+    <n v="5456.39"/>
+    <n v="50"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PivotTable1" cacheId="1" dataCaption="Values" compact="1" outline="1" subtotalTop="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PivotTable1" cacheId="1" dataCaption="Values" compact="1" outline="1" subtotalTop="1" updatedVersion="8" minRefreshableVersion="5" createdVersion="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" useAutoFormatting="1" itemPrintTitles="1" indent="0" outlineData="1" multipleFieldFilters="0">
   <location ref="G1:H6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">

</xml_diff>

<commit_message>
fix(pivots): reference generator — timeline style, scroll position and bounds from data (Task 2 fix round 4)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KTccUzeFqqMqTthqgFm9H
</commit_message>
<xml_diff>
--- a/tests/fixtures/xlsx-pivots/slicer-dark1.xlsx
+++ b/tests/fixtures/xlsx-pivots/slicer-dark1.xlsx
@@ -840,14 +840,14 @@
     <pivotTable tabId="2" name="PivotTable1"/>
   </pivotTables>
   <state minimalRefreshVersion="6" lastRefreshVersion="6" pivotCacheId="1" filterType="unknown">
-    <bounds startDate="2024-01-01T00:00:00" endDate="2026-01-01T00:00:00"/>
+    <bounds startDate="2024-01-01T00:00:00" endDate="2025-01-01T00:00:00"/>
   </state>
 </timelineCacheDefinition>
 </file>
 
 <file path=xl/timelines/timeline1.xml><?xml version="1.0" encoding="utf-8"?>
 <timelines xmlns="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <timeline name="Date" xr10:uid="{BCDD19F5-7DFF-6745-8336-A62734B2B7F9}" cache="NativeTimeline_Date" caption="Date" level="2" selectionLevel="2" scrollPosition="2025-06-22T00:00:00"/>
+  <timeline name="Date" xr10:uid="{BCDD19F5-7DFF-6745-8336-A62734B2B7F9}" cache="NativeTimeline_Date" caption="Date" level="2" selectionLevel="2" scrollPosition="2024-01-01T00:00:00"/>
 </timelines>
 </file>
 

</xml_diff>

<commit_message>
fix(pivots): reference generator — 12 Excel timeline styles, non-overlapping controls, visible slicer scroll and no-data (Task 2 fix round 5)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KTccUzeFqqMqTthqgFm9H
</commit_message>
<xml_diff>
--- a/tests/fixtures/xlsx-pivots/slicer-dark1.xlsx
+++ b/tests/fixtures/xlsx-pivots/slicer-dark1.xlsx
@@ -178,13 +178,13 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
+      <xdr:col>7</xdr:col>
       <xdr:colOff>787400</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:row>6</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>508000</xdr:colOff>
       <xdr:row>11</xdr:row>
       <xdr:rowOff>139700</xdr:rowOff>

</xml_diff>

<commit_message>
fix(pivots): reference generator — timeline and scrolled-slicer anchors sized from Excel captures (Task 2 fix round 6)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KTccUzeFqqMqTthqgFm9H
</commit_message>
<xml_diff>
--- a/tests/fixtures/xlsx-pivots/slicer-dark1.xlsx
+++ b/tests/fixtures/xlsx-pivots/slicer-dark1.xlsx
@@ -180,14 +180,14 @@
     <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>787400</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>508000</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>139700</xdr:rowOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:tsle="http://schemas.microsoft.com/office/drawing/2012/timeslicer" Requires="tsle">

</xml_diff>

<commit_message>
test(pivots): self-describing generated fixtures — Excel's own themes, styles link, no table-level subtotalTop
Generated workbooks now embed the theme Excel used for them (Office 2023 for table cases, the 2007-2010
theme for slicer/timeline cases), link xl/styles.xml, and drop the non-ECMA table-level subtotalTop
(Rulings AJ, AB). All 135 xml cases re-open clean in Excel 16.114 and were re-captured: colours are
unchanged, text now uses the declared Calibri 11 instead of Excel's fallback font, and timelines move
because their source dates now carry a date format. Three timeline handle checks fail against the new
references; they are fixed in the Task 12 follow-up.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KTccUzeFqqMqTthqgFm9H
</commit_message>
<xml_diff>
--- a/tests/fixtures/xlsx-pivots/slicer-dark1.xlsx
+++ b/tests/fixtures/xlsx-pivots/slicer-dark1.xlsx
@@ -622,7 +622,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PivotTable1" cacheId="1" dataCaption="Values" compact="1" outline="1" subtotalTop="1" updatedVersion="8" minRefreshableVersion="5" createdVersion="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" useAutoFormatting="1" itemPrintTitles="1" indent="0" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PivotTable1" cacheId="1" dataCaption="Values" compact="1" outline="1" updatedVersion="8" minRefreshableVersion="5" createdVersion="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" useAutoFormatting="1" itemPrintTitles="1" indent="0" outlineData="1" multipleFieldFilters="0">
   <location ref="G1:H6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField axis="axisRow" showAll="0">
@@ -753,9 +753,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -763,56 +763,177 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -821,16 +942,98 @@
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 

</xml_diff>